<commit_message>
chore(data-release): publish site data 2026-10-16 23:51:04 UTC
</commit_message>
<xml_diff>
--- a/diseases/d156/2026-2029.xlsx
+++ b/diseases/d156/2026-2029.xlsx
@@ -3846,6 +3846,399 @@
         </is>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>disease</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>D156</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>gastroenteritis</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Gastroenteritis</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>public_projection</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>NZ</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>D156</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Gastroenteritis</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>胃肠炎</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="N18" t="n">
+        <v>37</v>
+      </c>
+      <c r="O18" t="n">
+        <v>37</v>
+      </c>
+      <c r="R18" t="n">
+        <v>0.6997663725945767</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>wpp_computed</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>SER_NZ_GASTROENTERITIS_MONTHLY</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AO18" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP18" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ18" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS18" t="inlineStr">
+        <is>
+          <t>SER_NZ_GASTROENTERITIS_MONTHLY</t>
+        </is>
+      </c>
+      <c r="AT18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU18" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV18" t="inlineStr">
+        <is>
+          <t>phf_monthly</t>
+        </is>
+      </c>
+      <c r="AW18" t="inlineStr">
+        <is>
+          <t>New Zealand PHF Science Monthly Notifiable Diseases</t>
+        </is>
+      </c>
+      <c r="AX18" t="inlineStr">
+        <is>
+          <t>https://www.phfscience.nz/digital-library/</t>
+        </is>
+      </c>
+      <c r="AY18" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="AZ18" t="inlineStr">
+        <is>
+          <t>phf_monthly</t>
+        </is>
+      </c>
+      <c r="BA18" t="inlineStr">
+        <is>
+          <t>New Zealand PHF Science Monthly Notifiable Diseases</t>
+        </is>
+      </c>
+      <c r="BB18" t="inlineStr">
+        <is>
+          <t>https://www.phfscience.nz/digital-library/</t>
+        </is>
+      </c>
+      <c r="BC18" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>disease</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>D156</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>gastroenteritis</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Gastroenteritis</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>source_series_observation</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>NZ</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>D156</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Gastroenteritis</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>胃肠炎</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>Bacterial</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>37</v>
+      </c>
+      <c r="O19" t="n">
+        <v>37</v>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>SER_NZ_GASTROENTERITIS_MONTHLY</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>SER_NZ_GASTROENTERITIS_MONTHLY</t>
+        </is>
+      </c>
+      <c r="W19" t="inlineStr">
+        <is>
+          <t>SRC_NZ_PHS</t>
+        </is>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>Gastroenteritis</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>case_notifications</t>
+        </is>
+      </c>
+      <c r="Z19" t="inlineStr">
+        <is>
+          <t>notification</t>
+        </is>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>monthly</t>
+        </is>
+      </c>
+      <c r="AB19" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="AC19" t="inlineStr">
+        <is>
+          <t>country:NZ:national</t>
+        </is>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="AE19" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>conditional</t>
+        </is>
+      </c>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>non_additive</t>
+        </is>
+      </c>
+      <c r="AH19" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="AI19" t="inlineStr">
+        <is>
+          <t>missing_is_unknown</t>
+        </is>
+      </c>
+      <c r="AJ19" t="inlineStr">
+        <is>
+          <t>NZ_PHS_current</t>
+        </is>
+      </c>
+      <c r="AK19" t="inlineStr">
+        <is>
+          <t>New Zealand PHF Science monthly source-defined gastroenteritis notifications.</t>
+        </is>
+      </c>
+      <c r="AM19" t="inlineStr">
+        <is>
+          <t>provisional; raw</t>
+        </is>
+      </c>
+      <c r="AN19" t="b">
+        <v>1</v>
+      </c>
+      <c r="AO19" t="inlineStr">
+        <is>
+          <t>series_registry</t>
+        </is>
+      </c>
+      <c r="AP19" t="inlineStr">
+        <is>
+          <t>single_series</t>
+        </is>
+      </c>
+      <c r="AQ19" t="inlineStr">
+        <is>
+          <t>parity</t>
+        </is>
+      </c>
+      <c r="AS19" t="inlineStr">
+        <is>
+          <t>SER_NZ_GASTROENTERITIS_MONTHLY</t>
+        </is>
+      </c>
+      <c r="AT19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU19" t="inlineStr">
+        <is>
+          <t>The public curve is read directly from one registered source series.</t>
+        </is>
+      </c>
+      <c r="AV19" t="inlineStr">
+        <is>
+          <t>phf_monthly</t>
+        </is>
+      </c>
+      <c r="AW19" t="inlineStr">
+        <is>
+          <t>New Zealand PHF Science Monthly Notifiable Diseases</t>
+        </is>
+      </c>
+      <c r="AX19" t="inlineStr">
+        <is>
+          <t>https://www.phfscience.nz/digital-library/</t>
+        </is>
+      </c>
+      <c r="AY19" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+      <c r="AZ19" t="inlineStr">
+        <is>
+          <t>phf_monthly</t>
+        </is>
+      </c>
+      <c r="BA19" t="inlineStr">
+        <is>
+          <t>New Zealand PHF Science Monthly Notifiable Diseases</t>
+        </is>
+      </c>
+      <c r="BB19" t="inlineStr">
+        <is>
+          <t>https://www.phfscience.nz/digital-library/</t>
+        </is>
+      </c>
+      <c r="BC19" t="inlineStr">
+        <is>
+          <t>web</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3879,7 +4272,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
+          <t>2026-09-01</t>
         </is>
       </c>
     </row>
@@ -3962,7 +4355,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10">
@@ -3972,7 +4365,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11">
@@ -3992,7 +4385,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="13">
@@ -4024,7 +4417,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>312</v>
+        <v>349</v>
       </c>
     </row>
     <row r="16">

</xml_diff>